<commit_message>
Week 3: 7 lenders, intent fixes, 89% hit rate — remove .env from tracking
</commit_message>
<xml_diff>
--- a/data/Metadata/QuestionBank.xlsx
+++ b/data/Metadata/QuestionBank.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="632">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1097,31 +1097,796 @@
     <t xml:space="preserve">No. CFAL has no Low Doc option; documentation requirements scale up with transaction size, and full financial statements are required at every band.</t>
   </si>
   <si>
+    <t xml:space="preserve">ANG-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What are the qualifying criteria for Angle's $400k Low Doc program?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle's $400k Low Doc requires 3+ years ABN &amp; GST registered, a credit score of 600+ (Corporate &amp; Individual, Veda 1.1), a minimum 12-month Asset Finance Credit Reference from Angle or a Tier 1/Tier 2 provider, a max transaction size of $400k, property backing (spousal property accepted), asset types Primary &amp; Secondary, max EOT of Primary 25 years and Secondary 15 years, and ATO Portals for $250k+.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_400k_low_doc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which applicants and assets are excluded from Angle's $400k Low Doc program?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The $400k Low Doc program excludes sole traders, tertiary assets, prime movers, and buses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum loan and deposit under Angle's Start-Up product?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle's Start-Up product allows loans to a maximum of $150,000 (including brokerage), with a 20% deposit required on all applications. The business must be operating a minimum of 3 months and actively trading, with previous industry experience required.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_start_up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What entity types qualify for Angle's Prime Movers product, and is Low Doc available?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Movers is restricted to Company &amp; Trust only — no sole traders or individual partnerships. Low Doc is not an option for prime movers, because bank statements or financials plus ATO portals are required; they can be done under Mid Doc or Full Doc only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_prime_movers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Angle accept spousal property, and what deposit do non-property owners pay?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes — spousal property is accepted as asset backed, supported by a marriage certificate, Medicare card or joint utility bill. Non-property owners require a 20% deposit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_property_and_deposits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is Angle's establishment fee and maximum brokerage?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle's establishment fee (dealer or private sale) is $649, financed into the loan or direct debit at settlement. The account keeping fee is $4.95 monthly or $1 weekly. Maximum brokerage is up to 8% (incl GST), and there is no rate loading for commission up to 8%. An origination fee of up to $1,400 (incl GST) may be capitalised within the loan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_fees_brokerage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How does a customer's credit score determine total exposure at Angle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At Angle, credit score determines total exposure: a score of 500 allows under $150,000; 550 allows under $250,000; and 650 allows over $250,000. Large ticket deals over $500,000+ have credit score flexibility — scores under 650 can be considered with financial assessment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_loan_structure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Angle finance taxi or Uber drivers?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Taxi &amp; Uber drivers are on Angle's not-accepted applicants list. Angle also declines applicants with credit scores below 500, financial defaults on credit files (except telco or utilities paid up to $2,500), and credit files under 12 months old.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_exclusions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When does Angle require a Certificate of Currency, and how are private sales inspected?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle requires a Certificate of Currency for assets over $100k. Private sales require inspection via Verimoto, Redbook, Olasio or a broker inspection, and must have current and active registration. Angle conducts a satisfactory PPSR, and all existing PPSR encumbrances on used cars must be removed prior to settlement.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_settlement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum balloon on an Angle loan over a 60-month term?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The maximum balloon on a 60-month Angle loan is 30% (it is 40% at both 36 and 48 months). Assets at EOT 25 years (primary) and EOT 15 years (secondary) are 0% balloon only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What credit score does Angle require for Mid Doc, and what bank statements are needed?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle's Mid Doc (under $500k) requires a credit score of 650+ (Individual &amp; Corporate, Veda 1:1). It requires 6 months bank statements showing no dishonoured payments for financial obligations, a maximum of 1 non-financial dishonour, average monthly revenue of $20,000 across the 6-month period, and an average running balance of at least 10% of monthly revenue. ATO Portals are required for $250k+.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_doc_types</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is Angle's headline rate for an 8+ year ABN, 4+ year GST customer buying primary assets?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For a customer with 8+ year ABN and 4+ year GST buying primary assets (new assets, YOM 2023) with a strong credit score, the rate is 7.79% property backed and 8.79% non-property backed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle_interest_rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What ABN age and credit score does Angle require for Prime Movers, and what loading applies?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prime Movers requires a minimum 5 years ABN &amp; GST (business continuity), a strong credit score of 600+, property backing (spousal accepted), and a comparable asset finance credit reference. A 1% rate loading applies to standard primary asset rates. Maximum asset age is up to EOT 20 years.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What bank statement history does Angle's Start-Up product require?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start-Up requires a minimum of 6 months bank statements, unless the ABN has been trading for less than 6 months. The statements must demonstrate serviceability, show clean conduct with no overdraws, dishonours, debt collection payments, superannuation withdrawals or ATO payment arrangements, and support an average bank balance over the last 3 months of at least 10%–20% of the loan amount.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What does Angle's Full Doc require for a transaction over $1 million?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For transactions over $1 million, Angle's Full Doc requires FY2024 + FY2023 accountant-prepared financials only, a Commitment Schedule, current ATO portal statements (last 12 months good payment history), a detailed business background plus list of major clients, an Aged Debtor + Creditor listing, and cashflow projections (if available).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum loan term Angle offers on a primary motor vehicle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle offers up to 84 months on a primary motor vehicle (36–84 months). A 1% rate loading is applicable for terms over 60 months, and the customer must be property backed to qualify.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is Angle's rate for a prime mover?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle's Prime Movers start from 9.39% per the rate card (the prime movers flyer cites 8.99%). A 1% rate loading applies to standard primary asset rates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum motor vehicle finance amount under Angle's Low Doc?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under Low Doc, motor vehicles are capped at $100k for exposures under $100k, and $200k for exposures of $100k–$250k. The motor vehicle maximum asset price is $250k. Mid Doc allows motor vehicles up to $250k.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What proof of property ownership does Angle require?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle requires a rates notice for proof of property ownership, dated within the last 3 months or provided alongside a recent utility bill. Spousal property requires a marriage certificate, Medicare card or joint utility bill as evidence of relationship.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can an applicant with a paid financial default get finance from Angle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Financial defaults on credit files — whether paid or unpaid — are not accepted, with the only exception being telco or utility defaults paid up to $2,500.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can a business with an ABN under 2 years get finance from Angle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes. Angle's Start-Up product is designed for new business owners with an ABN under 2 years, provided the business has been operating a minimum of 3 months and actively trading, with a 20% deposit and 550+ credit score.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can a sole trader finance a prime mover with Angle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Angle's Prime Movers product is Company &amp; Trust only — sole traders and individual partnerships are explicitly excluded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can a mortgage statement in a spouse's name be used as a credit reference at Angle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Mortgage statements must be in the applicant's name — spouse's mortgage statements are not accepted. The loan must have been running 6+ months with no missed repayments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Angle charge a rate loading for brokerage?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Angle applies no rate loading for commission up to 8%. Private sales, business continuity and property in a spouse's name also attract no rate loading.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANG-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Angle apply a rate loading to private sales?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Angle explicitly applies no rate loading for private sales. The prime movers product also confirms there is no rate loading for private sales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is Metro's prime rate for a passenger vehicle under 5 years old?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro's 8.35% prime rate applies to passenger and commercial vehicles under 12t GVM, up to 5 years old, financed above $20k on a dealer sale, over a 24–60 month term. Amounts between $10k and $20k are priced at 9.15%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_interest_rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What loadings does Metro apply for older assets and private sales?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro adds 0.75% for assets older than 5 years at the beginning of term, 1.50% for assets older than 10 years at end of term, 0.25% for private sale, 0.75% for sale/hire backs, 2% to the wheeled equipment rate for other equipment, and 1% on the vehicle streamlined non-property product.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What deposit does Metro require for a non-property backed passenger vehicle loan?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For non-property backed applicants (motor vehicles only), Metro caps the loan at $100,000, permits dealer sale only, and requires a 30% deposit. Maximum Metro exposure for this category is $100,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_passenger_vehicle_streamlined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What Metro exposure applies to a customer with 24 months of good repayment history?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A customer with 24 months of good repayment history with Metro can reach a maximum Metro exposure of $750,000 (including existing Metro exposure). New Metro customers are capped at $250,000, and customers with 12 months good repayment history at $500,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are prime movers eligible under Metro's Trucks, Trailers &amp; Wheeled Equipment streamlined product?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Metro's Trucks, Trailers &amp; Wheeled Equipment streamlined product covers medium and heavy commercial vehicles above 3.5t GVM but explicitly excludes prime movers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_trucks_trailers_streamlined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What GST registration and farm size does Metro require under the Agri streamlined product?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro's Agri streamlined product requires the business to be GST registered for more than 5 years, to be a genuine primary producer, and to have a minimum farm size of 40 hectares. Maximum term is 60 months.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_agri_streamlined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can Metro finance equipment under the Other Equipment streamlined product via private sale?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. The Other Equipment streamlined product must be from a recognised supplier — no private sale or sale/hire back is permitted. The asset must be no older than 3 years and serial numbered, with a maximum loan of $100,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_other_equipment_streamlined</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under Metro's Replacement Policy, how long must the contract being replaced have run?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contracts being replaced must have run for a minimum of 36 months. The new loan amount must not exceed 125% of the original loan amount of the contract being replaced, or the proposed monthly repayment must not exceed 125% of the monthly repayment being replaced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_replacement_policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What rate discount and loan term apply to MetroEco electric trucks?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MetroEco electric trucks receive a 1% MetroEco rate discount. They must be brand new assets only, dealer sale, battery electric trucks 3.5t GVM and above, property owners only, up to $250,000 for new customers or $300,000 with 12 months good repayment history. Maximum transaction size is $600,000 with full financials, and maximum electric truck exposure is $700,000. Biofuel and hybrid are excluded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_eco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is Metro's maximum lending in a 12-month period under streamlined products?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro caps streamlined lending at a maximum of $500,000 in a 12 month period. Sale/hire back is not permitted under streamlined products, and satisfactory Equifax is required on applicants and guarantors.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_exclusions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum loan for a new Metro customer buying a truck, and what is the private sale cap?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A new Metro customer can borrow up to $250,000 (dealer and private sale) for trucks and trailers, rising to $300,000 with 12 months good repayment history with Metro. The maximum transaction size for private sales is $250,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum asset age at end of term for a Metro passenger vehicle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under the Passenger Vehicle streamlined product (&lt;3.5t GVM), the asset must be no older than 12 years at end of term. Trucks, trailers and wheeled equipment allow up to 15 years at end of term.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum loan under Metro's Replacement Policy for medium and heavy commercial vehicles?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro's Replacement Policy allows $300,000 for medium &amp; heavy commercial (excludes prime movers), trailers and wheeled equipment on dealer sales; $150,000 for passenger vehicles and light commercial; and a maximum transaction size of $250,000 for private sales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What loan term does MetroEco offer for a commercial electric vehicle?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A commercial MetroEco electric vehicle has a 60-month loan term with a maximum EOT of 5 years, for up to $91,387.00 on vehicles, new or demo, from a dealer. Consumers get 84 months (max EOT 7 years) and novated is 60 months.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum loan for agricultural implements under Metro's Agri product?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implements / Tertiary Equipment are capped at $150,000 maximum (dealer/private sale) with a $10,000 minimum, for both new and existing Metro customers. Primary agricultural equipment allows $250,000, rising to $300,000 with 12 months good repayment history.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How does brokerage above 4% affect a Metro rate?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro's advertised rates apply for brokerage up to 4%. Above 4.0%, add 0.5% to the base rate for every 1% of brokerage.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What fees does Metro charge?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro charges a minimum fee of $275 and a maximum of $450, excluding split 50/50.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When must a contract be to qualify for Metro's Balloon/Residual Refinance product?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The account being replaced must be in its final 12 months. The product covers motor vehicles and wheeled equipment only, and prime movers are included. No inspection is required.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">metro_balloon_refinance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Metro finance dairy and irrigation equipment under the Agri product?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Dairy equipment and irrigation equipment are both on Metro's Agri non-eligible list, along with sheds, silos, yards, testing and measurement equipment, bikes &amp; ATVs, and forestry industry assets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What GST registration does Metro require for the passenger vehicle streamlined product?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro requires the business to be GST registered 2 years continuously for the passenger vehicle streamlined product.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does Metro allow sale and hire back under its streamlined products?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. Sale/hire back is not permitted under Metro's streamlined products. A 0.75% sale/hire back loading appears on the rate sheet for non-streamlined deals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can Metro finance IT and audio-visual equipment under the Other Equipment product?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. IT, AV, telephony and printing equipment are explicitly non-eligible under Metro's Other Equipment streamlined product, along with fixtures &amp; fittings, retail/health/beauty/fitness, mining, and intangible assets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does MetroEco finance hybrid vehicles?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. MetroEco electric trucks explicitly exclude biofuel powered or hybrid vehicles. MetroEco electric vehicle eligibility requires the vehicle be solely powered by electricity and use an external electrical plug to charge the battery.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are taxi and Uber applications accepted by Metro?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, but with restrictions: taxi / Uber / ride share applications have a maximum customer exposure of $250,000 and must be property backed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MET-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is Metro's maximum single asset and customer exposure?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro's rate sheet states single assets up to $1m and customer exposure up to $2m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flexi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the flexipremium rate for a primary asset funded between $100,001 and $500,000?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexipremium prices primary assets at 7.30% for amounts funded between $100,001 and $500,000 (also 7.30% for $50,000–$100,000). Secondary assets in that band are 8.19%. Amounts of $500,001+ require contacting a flexicommercial BDM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexi_flexipremium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What time in business does flexipremium require, and are sole traders eligible?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexipremium requires asset-backed applicants to have ABN and GST registration for a minimum of 4 years, and non-asset-backed applicants a minimum of 8 years. Eligible business structures are Companies, Trusts and Partnerships — sole traders are excluded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is flexicommercial's standard base rate for a primary asset above $150,001?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For primary assets of $150,001+, flexicommercial's standard base rate is 8.10% (ex brokerage). Secondary is 8.35% and tertiary is 11.35% in the same band.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexi_standard_rates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What add-ons does flexicommercial apply to its standard base rates?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexicommercial adds 1.0% for prime movers (excluding tippers, agitators, rigid bodies), assets 11–15 years old at end of term, terms under 24 months, and private sales and refinances. It adds 1.25% for non-asset-backed customers and terms over 60 months. It adds 2.0% for assets over 15 to 20 years old at end of term.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What are flexicommercial's maximum exposures by asset class?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexicommercial's Credit Matrix allows Primary Assets up to $750K (individual transactions up to $500K), Secondary Assets up to $500K (individual transactions up to $300K), and Tertiary Assets up to $300K (individual transactions up to $300K).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexi_credit_matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does flexicommercial fund SUVs or passenger cars?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. flexicommercial explicitly does not fund SUVs or passenger cars, including rental car businesses. It also does not fund photocopiers, MFDs or scaffolding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexi_asset_categories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How old can a primary asset be at end of term at flexicommercial?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary assets must not exceed 20 years at end of term, with trailers permitted up to 30 years. Secondary assets can be up to 7 years old at end of term.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum transaction size and repayment increase under flexireplacement?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexireplacement allows a maximum transaction size / aggregated exposure of $500K (including existing matrix exposure). The proposed repayment must not exceed 125% of that being replaced. It covers primary assets only, with dealer or private sales acceptable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexi_replacement_policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under flexireplacement, what conditions apply to the facility being replaced?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The facility to be replaced must be with an approved lender, and either current or paid in full within the last three months, after having been established for 18 months or more. Borrowing and guarantee parties on the old and new facility must be identical, and settlement of the new facility must occur within 90 days of the expiry of the old facility.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is flexicommercial's establishment fee?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexicommercial charges an establishment fee of $495 on all products, rising to $745 for private sales and refinances. The minimum deal size is $10,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexi_fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is flexicommercial's maximum brokerage on a deal of $60,000?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For deals of $50,000 or more, maximum brokerage is 6%, and 0.5% is added to the base rate for every 1% of brokerage charged above 4% (up to 6%). Deals under $50,000 allow up to 8% brokerage, with the escalation starting above 5%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How old can assets be under flexipremium?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Under flexipremium, primary assets can be up to 5 years old (Contract Road Transport/Logistics businesses operating 5 or more trucks can be considered), and secondary assets up to 2 years old. Both new and used assets are eligible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How can a flexicommercial customer increase their exposure to $750K?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary Assets Only: after 18 payments have been made on either the flexicommercial contract or an asset finance contract with an approved lender (minimum contract amount $250K, with a statement showing perfect conduct), applications can be considered to take combined exposure to a maximum of $750K, with individual transactions to a maximum of $500K.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What brokerage applies to a flexicommercial mid-term refinance?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brokerage on a mid-term refinance is limited to 1.0%. The customer must be at least 12 months into the term of the current contract, and the deal is refinanced at net book value with no early termination costs. Terms of up to 5 years are considered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexi_refinance_products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How does a flexipremium Low Start Loan work?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Low Start Loan lets the business start their term paying 50% repayments for the first 3 months, then catch that up gradually over time. Conditions: the customer must qualify for flexipremium, have no cashflow lenders on file (e.g. Prospa, Moula), and must have an existing commercial asset finance facility with an approved lender.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What ABN and GST duration does flexicommercial's Credit Matrix require?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Credit Matrix requires ABN greater than 2 years and GST registered greater than 2 years, with asset backing (sufficient equity) or a 20% deposit assessed on the proposed aggregate exposure, not just the new transaction.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum exposure for IT assets at flexicommercial?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All IT assets are tertiary assets with a maximum exposure of $50K; full doc is acceptable for amounts over $50K. The same $50K cap applies to renewable energy and temporary fencing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is flexicommercial's maximum loan term?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The maximum term is 7 years on primary assets up to 3 years old; for all other assets the maximum term is 5 years. Terms over 60 months attract a 1.25% add-on.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are sole traders eligible at flexicommercial?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sole traders are covered by the standard Credit Matrix (which applies to Companies, Trusts, Partnerships and Sole Traders), but they are excluded from flexipremium, which is limited to Companies, Trusts and Partnerships.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexi_exclusions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can flexireplacement be used for balloon refinances?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes. flexireplacement can be used for balloon refinances up to $500K, with an inspection and valuation required if the amount exceeds $300K.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does flexicommercial finance passenger cars for a rental car business?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. flexicommercial explicitly does not fund SUVs or passenger cars, and this includes rental car businesses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the maximum brokerage on a flexipremium deal?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum brokerage on flexipremium deals is 3%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do transport operators need to be asset backed at flexicommercial?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes. Asset backing is a requirement for all transport operator/subcontractor transactions — borrowers and guarantors must be asset backed with sufficient equity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is flexicommercial's minimum deal size?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flexicommercial's minimum deal size is $10,000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLX-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How does flexicommercial classify medical and dental equipment?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medical / dental / laboratory equipment is classified as a secondary asset at flexicommercial. Secondary assets can be up to 7 years old at end of term.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CMAP 2026 — Question Bank</t>
   </si>
   <si>
     <t xml:space="preserve">Purpose</t>
   </si>
   <si>
-    <t xml:space="preserve">Benchmark set of gold-standard questions across the four lender policy sets.</t>
+    <t xml:space="preserve">Benchmark set of gold-standard questions across the seven lender policy sets.</t>
   </si>
   <si>
     <t xml:space="preserve">Scope</t>
   </si>
   <si>
-    <t xml:space="preserve">100 questions total — 25 per lender (Resimac, BFS, Westpac, CFAL).</t>
+    <t xml:space="preserve">175 questions total — 25 per lender (Resimac, BFS, Westpac, CFAL, Angle, Metro, Flexi).</t>
   </si>
   <si>
     <t xml:space="preserve">Gold standard</t>
   </si>
   <si>
-    <t xml:space="preserve">Every question here carries its 4/4 reference answer (the gold-standard answer).</t>
+    <t xml:space="preserve">Every question carries its 4/4 reference answer (the gold-standard answer).</t>
   </si>
   <si>
     <t xml:space="preserve">Grounding</t>
   </si>
   <si>
-    <t xml:space="preserve">All answers are derived verbatim from the enhanced *_chunks.md policy files.</t>
+    <t xml:space="preserve">All answers derived verbatim from the enhanced *_chunks.md policy files.</t>
   </si>
   <si>
     <t xml:space="preserve">Columns</t>
@@ -1142,10 +1907,16 @@
     <t xml:space="preserve">ELIGIBILITY, PRICING, LOAN_LIMITS, DOCUMENTATION, ASSET_ELIGIBILITY, EXCLUSIONS, SETTLEMENT, SPECIAL_PROGRAMS, FEES.</t>
   </si>
   <si>
-    <t xml:space="preserve">Chunk IDs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Match the stable chunk_id keys used by the vector DB — usable as retrieval-eval targets.</t>
+    <t xml:space="preserve">ID prefixes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RES / BFS / WBC / CFA / ANG / MET / FLX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golden rule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every Source Chunk ID resolves to a row in Metadata.csv (62 chunks).</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1978,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1223,25 +1994,43 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8EEF7"/>
-        <bgColor rgb="FFEAF3EA"/>
+        <bgColor rgb="FFE8F4FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEAF3EA"/>
+        <bgColor rgb="FFE8F4FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBEAEC"/>
+        <bgColor rgb="FFF2EAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3EEF8"/>
+        <bgColor rgb="FFF2EAF6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2E8"/>
+        <bgColor rgb="FFFBEAEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F4FA"/>
         <bgColor rgb="FFE8EEF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFBEAEC"/>
+        <fgColor rgb="FFF2EAF6"/>
         <bgColor rgb="FFF3EEF8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF3EEF8"/>
-        <bgColor rgb="FFE8EEF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -1294,7 +2083,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1320,6 +2109,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1360,12 +2161,12 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFF3EEF8"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFEAF3EA"/>
-      <rgbColor rgb="FFE8EEF7"/>
+      <rgbColor rgb="FFFFF2E8"/>
+      <rgbColor rgb="FFE8F4FA"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1379,13 +2180,13 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFF3EEF8"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFEAF3EA"/>
+      <rgbColor rgb="FFE8EEF7"/>
       <rgbColor rgb="FFFBEAEC"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFF2EAF6"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1587,7 +2388,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G176"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
@@ -3920,6 +4721,1731 @@
       </c>
       <c r="G101" s="2" t="s">
         <v>282</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B102" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E102" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="G102" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="G103" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B104" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="G104" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B105" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="G105" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="B106" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="G106" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="B107" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="G107" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="B108" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="B110" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E110" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="G110" s="2" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="G111" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="B112" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="G112" s="2" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="B113" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="B114" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="B115" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B116" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="F116" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B117" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B118" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="B119" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="B120" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="G120" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B121" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="B122" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B123" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B124" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="B125" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="F125" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="B126" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="B127" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="G127" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="B128" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="B129" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="B130" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="G130" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="B131" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="B132" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="B134" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="B135" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="B137" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="G137" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="B138" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="G138" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="B139" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="G139" s="2" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A140" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="B140" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="F140" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A141" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="B142" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="F142" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="B143" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="F143" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="G143" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="B144" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="F144" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="G144" s="2" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B145" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D145" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E145" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="F145" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="G145" s="2" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="B146" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="F146" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="G146" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="F147" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="G147" s="2" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="B148" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="F148" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="G148" s="2" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="B149" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D149" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="F149" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="G149" s="2" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="B150" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="G150" s="2" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="B151" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D151" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="F151" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="G151" s="2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="B152" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D152" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="F152" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="G152" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="B153" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D153" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="F153" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="G153" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="B154" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D154" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="F154" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="G154" s="2" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="B155" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="F155" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="G155" s="2" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="B156" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E156" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="F156" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="G156" s="2" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="B157" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="F157" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="G157" s="2" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="158" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="B158" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E158" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="F158" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="G158" s="2" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="B159" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C159" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E159" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>557</v>
+      </c>
+      <c r="G159" s="2" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="B160" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C160" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E160" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="F160" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="G160" s="2" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="161" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="B161" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C161" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E161" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="F161" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="G161" s="2" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="162" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="B162" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C162" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D162" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E162" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="F162" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="G162" s="2" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="163" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="B163" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E163" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="F163" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G163" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="B164" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="F164" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="G164" s="2" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="165" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="B165" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C165" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D165" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E165" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="F165" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="G165" s="2" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="B166" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C166" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D166" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E166" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="F166" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="G166" s="2" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="B167" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C167" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D167" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E167" s="2" t="s">
+        <v>583</v>
+      </c>
+      <c r="F167" s="2" t="s">
+        <v>584</v>
+      </c>
+      <c r="G167" s="2" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="B168" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C168" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E168" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="F168" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="G168" s="2" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="B169" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="F169" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="G169" s="2" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="B170" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C170" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E170" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="F170" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="G170" s="2" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="B171" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C171" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E171" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="F171" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="G171" s="2" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="2" t="s">
+        <v>598</v>
+      </c>
+      <c r="B172" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E172" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="F172" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="G172" s="2" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="B173" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C173" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E173" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="F173" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="G173" s="2" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="B174" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E174" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="F174" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="G174" s="2" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="B175" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C175" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D175" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E175" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="F175" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="G175" s="2" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="B176" s="9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E176" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="F176" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="G176" s="2" t="s">
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -3938,80 +6464,88 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="96"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>358</v>
+      <c r="A1" s="10" t="s">
+        <v>613</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="s">
-        <v>359</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>360</v>
+      <c r="A3" s="11" t="s">
+        <v>614</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>615</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>361</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>362</v>
+      <c r="A4" s="11" t="s">
+        <v>616</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>617</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="s">
-        <v>363</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>364</v>
+      <c r="A5" s="11" t="s">
+        <v>618</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>619</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="s">
-        <v>365</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>366</v>
+      <c r="A6" s="11" t="s">
+        <v>620</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>621</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>367</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>368</v>
+      <c r="A7" s="11" t="s">
+        <v>622</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>623</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>369</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>370</v>
+      <c r="A8" s="11" t="s">
+        <v>624</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>625</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>371</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>372</v>
+      <c r="A9" s="11" t="s">
+        <v>626</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>374</v>
+      <c r="A10" s="11" t="s">
+        <v>628</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>630</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>